<commit_message>
Fix 02_Solver.xlsx: remove invalid formula string and Unicode from IF formulas
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-10/02_Solver.xlsx
+++ b/rFLA300/chapter-10/02_Solver.xlsx
@@ -649,7 +649,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Chapter 10 — Solver</t>
+          <t>Chapter 10 - Solver</t>
         </is>
       </c>
     </row>
@@ -675,9 +675,9 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>1. OBJECTIVE CELL — the cell you want to maximize, minimize, or set to a specific value.
-2. VARIABLE CELLS — the cells Solver can change to reach the objective.
-3. CONSTRAINTS — rules that limit what values the variable cells can take.</t>
+          <t>1. OBJECTIVE CELL -- the cell you want to maximize, minimize, or set to a specific value.
+2. VARIABLE CELLS -- the cells Solver can change to reach the objective.
+3. CONSTRAINTS -- rules that limit what values the variable cells can take.</t>
         </is>
       </c>
     </row>
@@ -690,8 +690,8 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Data tab  →  Analyze group  →  Solver
-(If Solver is missing: File → Options → Add-ins → Manage: Excel Add-ins → Go → check Solver Add-in)</t>
+          <t>Data tab  -&gt;  Analyze group  -&gt;  Solver
+(If Solver is missing: File -&gt; Options -&gt; Add-ins -&gt; Manage: Excel Add-ins -&gt; Go -&gt; check Solver Add-in)</t>
         </is>
       </c>
     </row>
@@ -704,10 +704,10 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>• Maximize profit given limited resources (labor, materials, budget)
-• Minimize cost while meeting demand requirements
-• Find the best product mix
-• Schedule staff efficiently</t>
+          <t>- Maximize profit given limited resources (labor, materials, budget)
+- Minimize cost while meeting demand requirements
+- Find the best product mix
+- Schedule staff efficiently</t>
         </is>
       </c>
     </row>
@@ -720,8 +720,8 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Sheet  Production_Mix  — maximize profit with two products and three resource constraints.
-Sheet  Diet_Problem    — minimize cost while meeting nutritional requirements.</t>
+          <t>Sheet  Production_Mix  -- maximize profit with two products and three resource constraints.
+Sheet  Diet_Problem    -- minimize cost while meeting nutritional requirements.</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Solver Practice — Production Mix Optimization</t>
+          <t>Solver Practice - Production Mix Optimization</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
     <row r="6" ht="24" customHeight="1">
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Product Information (Fixed Data — do not change)</t>
+          <t>Product Information (Fixed Data - do not change)</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>≤ Available</t>
+          <t>&lt;= Available</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>≤ Available</t>
+          <t>&lt;= Available</t>
         </is>
       </c>
     </row>
@@ -876,14 +876,14 @@
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>≤ Available</t>
+          <t>&lt;= Available</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Min. Demand — Desk Lamp</t>
+          <t>Min. Demand - Desk Lamp</t>
         </is>
       </c>
       <c r="C12" s="10" t="n"/>
@@ -893,14 +893,14 @@
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>≥ Min</t>
+          <t>&gt;= Min</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Min. Demand — Floor Lamp</t>
+          <t>Min. Demand - Floor Lamp</t>
         </is>
       </c>
       <c r="C13" s="10" t="n"/>
@@ -910,14 +910,14 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>≥ Min</t>
+          <t>&gt;= Min</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Max. Demand — Desk Lamp</t>
+          <t>Max. Demand - Desk Lamp</t>
         </is>
       </c>
       <c r="C14" s="10" t="n"/>
@@ -927,14 +927,14 @@
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>≤ Max</t>
+          <t>&lt;= Max</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Max. Demand — Floor Lamp</t>
+          <t>Max. Demand - Floor Lamp</t>
         </is>
       </c>
       <c r="C15" s="10" t="n"/>
@@ -944,7 +944,7 @@
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>≤ Max</t>
+          <t>&lt;= Max</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="E19" s="18" t="inlineStr">
         <is>
-          <t>Start value — Solver will find the optimal quantity</t>
+          <t>Start value - Solver will find the optimal quantity</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E20" s="18" t="inlineStr">
         <is>
-          <t>Start value — Solver will find the optimal quantity</t>
+          <t>Start value - Solver will find the optimal quantity</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
     <row r="22" ht="24" customHeight="1">
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Objective Function  (Cell to Maximize — Result Cell)</t>
+          <t>Objective Function  (Cell to Maximize - Result Cell)</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Formula</t>
+          <t>Formula Reference</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1049,9 +1049,10 @@
           <t>Total Profit</t>
         </is>
       </c>
-      <c r="C24" s="20">
-        <f>C19*C8 + C20*C8   (Desk Profit + Floor Profit)</f>
-        <v/>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>Desk Lamps x $45  +  Floor Lamps x $65</t>
+        </is>
       </c>
       <c r="D24" s="21">
         <f>(C19*45)+(C20*65)</f>
@@ -1062,7 +1063,7 @@
     <row r="26" ht="24" customHeight="1">
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>Resource Usage  (Calculated — used in Constraints)</t>
+          <t>Resource Usage  (Calculated - used in Constraints)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1112,7 @@
         <v/>
       </c>
       <c r="F28" s="24">
-        <f>IF(C28&gt;D28,"OVER LIMIT ⚠","OK ✓")</f>
+        <f>IF(C28&gt;D28,"OVER LIMIT","OK")</f>
         <v/>
       </c>
     </row>
@@ -1133,7 +1134,7 @@
         <v/>
       </c>
       <c r="F29" s="24">
-        <f>IF(C29&gt;D29,"OVER LIMIT ⚠","OK ✓")</f>
+        <f>IF(C29&gt;D29,"OVER LIMIT","OK")</f>
         <v/>
       </c>
     </row>
@@ -1155,7 +1156,7 @@
         <v/>
       </c>
       <c r="F30" s="24">
-        <f>IF(C30&gt;D30,"OVER LIMIT ⚠","OK ✓")</f>
+        <f>IF(C30&gt;D30,"OVER LIMIT","OK")</f>
         <v/>
       </c>
     </row>
@@ -1170,7 +1171,7 @@
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>1.  Data tab  →  Solver  (if missing, enable via File → Options → Add-ins → Solver Add-in).</t>
+          <t>1.  Data tab  -&gt;  Solver  (if missing, enable via File -&gt; Options -&gt; Add-ins -&gt; Solver Add-in).</t>
         </is>
       </c>
     </row>
@@ -1198,63 +1199,63 @@
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C28 &lt;= D28   (Assembly Labor used ≤ available)</t>
+          <t xml:space="preserve">    - C28 &lt;= D28   (Assembly Labor used &lt;= available)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C29 &lt;= D29   (Finishing Labor used ≤ available)</t>
+          <t xml:space="preserve">    - C29 &lt;= D29   (Finishing Labor used &lt;= available)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C30 &lt;= D30   (Materials used ≤ available)</t>
+          <t xml:space="preserve">    - C30 &lt;= D30   (Materials used &lt;= available)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C19 &gt;= 10    (Min demand: Desk Lamp)</t>
+          <t xml:space="preserve">    - C19 &gt;= 10    (Min demand: Desk Lamp)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C20 &gt;= 5     (Min demand: Floor Lamp)</t>
+          <t xml:space="preserve">    - C20 &gt;= 5     (Min demand: Floor Lamp)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C19 &lt;= 60    (Max demand: Desk Lamp)</t>
+          <t xml:space="preserve">    - C19 &lt;= 60    (Max demand: Desk Lamp)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C20 &lt;= 40    (Max demand: Floor Lamp)</t>
+          <t xml:space="preserve">    - C20 &lt;= 40    (Max demand: Floor Lamp)</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="B44" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C19 = integer  (you cannot produce a fraction of a lamp)</t>
+          <t xml:space="preserve">    - C19 = integer  (you cannot produce a fraction of a lamp)</t>
         </is>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="B45" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C20 = integer</t>
+          <t xml:space="preserve">    - C20 = integer</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1281,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="23">
+    <mergeCell ref="B4:F4"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B46:F46"/>
     <mergeCell ref="B22:F22"/>
@@ -1331,7 +1333,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Solver Challenge — Minimum Cost Diet Problem</t>
+          <t>Solver Challenge - Minimum Cost Diet Problem</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1499,7 @@
     <row r="14" ht="24" customHeight="1">
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Decision Variables — Servings of Each Food (Solver Changes These)</t>
+          <t>Decision Variables - Servings of Each Food (Solver Changes These)</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1569,7 @@
     <row r="22" ht="24" customHeight="1">
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Objective — Total Daily Cost (Minimize This Cell)</t>
+          <t>Objective - Total Daily Cost (Minimize This Cell)</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1628,7 @@
         <v>50</v>
       </c>
       <c r="E27" s="24">
-        <f>IF(C27&gt;=D27,"✓ Met","✗ Not Met")</f>
+        <f>IF(C27&gt;=D27,"Met","Not Met")</f>
         <v/>
       </c>
     </row>
@@ -1644,7 +1646,7 @@
         <v>130</v>
       </c>
       <c r="E28" s="24">
-        <f>IF(C28&gt;=D28,"✓ Met","✗ Not Met")</f>
+        <f>IF(C28&gt;=D28,"Met","Not Met")</f>
         <v/>
       </c>
     </row>
@@ -1662,7 +1664,7 @@
         <v>20</v>
       </c>
       <c r="E29" s="24">
-        <f>IF(C29&gt;=D29,"✓ Met","✗ Not Met")</f>
+        <f>IF(C29&gt;=D29,"Met","Not Met")</f>
         <v/>
       </c>
     </row>
@@ -1680,7 +1682,7 @@
         <v>500</v>
       </c>
       <c r="E30" s="24">
-        <f>IF(C30&gt;=D30,"✓ Met","✗ Not Met")</f>
+        <f>IF(C30&gt;=D30,"Met","Not Met")</f>
         <v/>
       </c>
     </row>
@@ -1695,7 +1697,7 @@
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>1.  Open Solver: Data tab → Solver.</t>
+          <t>1.  Open Solver: Data tab -&gt; Solver.</t>
         </is>
       </c>
     </row>
@@ -1723,42 +1725,42 @@
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C27 &gt;= D27   (Protein ≥ 50 g)</t>
+          <t xml:space="preserve">    - C27 &gt;= D27   (Protein &gt;= 50 g)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C28 &gt;= D28   (Carbs ≥ 130 g)</t>
+          <t xml:space="preserve">    - C28 &gt;= D28   (Carbs &gt;= 130 g)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C29 &gt;= D29   (Fat ≥ 20 g)</t>
+          <t xml:space="preserve">    - C29 &gt;= D29   (Fat &gt;= 20 g)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C30 &gt;= D30   (Calories ≥ 500)</t>
+          <t xml:space="preserve">    - C30 &gt;= D30   (Calories &gt;= 500)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • C16:C20 &gt;= 0  (Cannot have negative servings)</t>
+          <t xml:space="preserve">    - C16:C20 &gt;= 0  (Cannot have negative servings)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="26" t="inlineStr">
         <is>
-          <t>5.  Solving Method:  GRG Nonlinear  (quantities don't have to be whole numbers).</t>
+          <t>5.  Solving Method:  GRG Nonlinear  (quantities do not have to be whole numbers).</t>
         </is>
       </c>
     </row>

</xml_diff>